<commit_message>
Add Denmark, operators (TSO/DSO/market clearing), Future-in-Europe, animations & richer cost explanation
- New deep-dive country: Denmark (Energinet TSO, DK1/DK2, Tarifmodel 3.0, elafgift, PSO abolished)
- Each country page now shows 'Who runs the grid & market': TSO(s) tile map, DSO landscape, day-ahead market-clearing operator (NEMO/SDAC/EUPHEMIA), price zones
- New 'Future in Europe' tab: SDAC, EUPHEMIA, 15-min MTU (live 30 Sep 2025), SIDC/IDA1-3, flow-based coupling, Nord Pool system price — cited (ENTSO-E/NEMO/Nord Pool)
- China updated for NDRC/NEA Doc 136/2025 (new-energy prices fully marketised) + coal capacity price
- Richer cost explanation: plain-English formulaIntro + animated 'anatomy of the bill' stacked-bar chart per country
- Animations via framer-motion (scroll reveal, animated bars); UI polish
- Excel workbook regenerated with Denmark

https://claude.ai/code/session_019Gbu6ZYe3PSRrb3yJdSZdx
</commit_message>
<xml_diff>
--- a/public/electricity-pricing-tutor.xlsx
+++ b/public/electricity-pricing-tutor.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Outputs" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Country_Germany" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Country_Sweden" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Country_China" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Country_Denmark" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Country_China" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="Depot_E">Inputs!$B$2</definedName>
@@ -583,17 +584,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -603,30 +604,34 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Country_China</t>
+          <t>Country_Denmark</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Albania</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>needs-research</t>
+          <t>deep-dive</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -634,12 +639,16 @@
           <t>2026-06-11</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Country_China</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Albania</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -663,7 +672,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -687,7 +696,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -711,7 +720,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -735,7 +744,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -759,7 +768,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Cyprus</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -783,7 +792,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Cyprus</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -807,7 +816,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -2772,6 +2781,388 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Denmark — truck-depot electricity tariff</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>A · Classification &amp; assumptions</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MV/HV (10-60 kV) business (C/B customer). Energy = Nord Pool spot, zone DK1 (west) or DK2 (east). TSO Energinet; DSO time-of-day tariff (Radius Tarifmodel 3.0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>B · Tariff components</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Legal basis</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Calculation</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Region variation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Spotpris (energy)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>energy</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Nord Pool day-ahead DK1/DK2</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>E x p_spot (zone-dependent)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Supplier &amp; zone</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Energinet systemtarif</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>grid-energy</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Energinet tariff reg.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>0.072 DKK/kWh (2026)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Energinet nettarif</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>grid-energy</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Energinet tariff reg.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>0.043 DKK/kWh (2026); +187 kr sub</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DSO nettarif (Tarifmodel 3.0)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>grid-energy</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>DSO; Forsyningstilsynet</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>ToU lav/hoj/spids; winter higher</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Each DSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Elafgift (electricity tax)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Lov om afgift af elektricitet</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>~0.008 DKK/kWh (2026 EU min); biz refund</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>PSO-tarif</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>levy</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Former Elforsyningsloven</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>0 (abolished end-2022)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Moms (VAT)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Momsloven</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>25% (recoverable)</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>C · Symbolic formulas</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>C_energy = E * p_spot (DK1/DK2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Energinet</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>C_energinet = E*0.115 + 187 = 230000 + sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>DSO grid</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>C_dso = sum_period(E_period * rate_period)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Electricity tax</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>C_elafgift = E*0.008 ~ 16000 (biz refund)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>C_preVAT = energy+energinet+dso+elafgift; x1.25 VAT (recoverable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>D · V2G / feed-in / export</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Export =&gt; producer/feed-in under Energinet+DSO; sold at ~spot; Energinet flexibility/balancing markets. Early V2G testbed (Parker) but no dedicated V2G tariff as of mid-2026; not modelled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>F · References — see the web app country page for full citation list</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B20:E20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>